<commit_message>
clean scripts study 2 publish
</commit_message>
<xml_diff>
--- a/0_data/three_challenges_codebook.xlsx
+++ b/0_data/three_challenges_codebook.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Clemens Lindner\Documents\GitHub\bigot_and_tolerant_personalites\0_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8460D08D-A1F1-41E0-A7FE-C45211640101}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37DCE64E-BDB4-495E-8802-753359BD9938}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-80" yWindow="-80" windowWidth="19360" windowHeight="11440" xr2:uid="{5059903E-ADBB-4520-B1A6-60D4EA1E22CC}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{5059903E-ADBB-4520-B1A6-60D4EA1E22CC}"/>
   </bookViews>
   <sheets>
     <sheet name="Study 1a" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1626" uniqueCount="711">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1648" uniqueCount="714">
   <si>
     <t>variable</t>
   </si>
@@ -2638,6 +2638,15 @@
   </si>
   <si>
     <t>1 = isced_1, 2 = isced_2, 3 = isced_2, 4 = isced_3, 5 = isced_4, 6 = isced_6, 7 = isced_7</t>
+  </si>
+  <si>
+    <t>factor</t>
+  </si>
+  <si>
+    <t>numeric</t>
+  </si>
+  <si>
+    <t>var_type</t>
   </si>
 </sst>
 </file>
@@ -7724,19 +7733,20 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4791DDA-356D-43C5-A405-960C4C715D9E}">
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="18.36328125" customWidth="1"/>
     <col min="2" max="2" width="15.36328125" customWidth="1"/>
     <col min="3" max="3" width="33.36328125" customWidth="1"/>
-    <col min="4" max="4" width="26.26953125" customWidth="1"/>
-    <col min="5" max="5" width="26.7265625" customWidth="1"/>
-    <col min="6" max="6" width="26.26953125" customWidth="1"/>
-    <col min="7" max="7" width="21.7265625" customWidth="1"/>
+    <col min="4" max="4" width="23.1796875" customWidth="1"/>
+    <col min="5" max="5" width="26.26953125" customWidth="1"/>
+    <col min="6" max="6" width="26.7265625" customWidth="1"/>
+    <col min="7" max="7" width="26.26953125" customWidth="1"/>
+    <col min="8" max="8" width="21.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>674</v>
       </c>
@@ -7747,22 +7757,25 @@
         <v>140</v>
       </c>
       <c r="D1" t="s">
+        <v>713</v>
+      </c>
+      <c r="E1" t="s">
         <v>676</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>675</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>687</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>512</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>251</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>514</v>
       </c>
@@ -7770,10 +7783,13 @@
         <v>514</v>
       </c>
       <c r="D2" t="s">
+        <v>711</v>
+      </c>
+      <c r="E2" t="s">
         <v>513</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:9">
       <c r="A3" t="s">
         <v>454</v>
       </c>
@@ -7781,10 +7797,13 @@
         <v>578</v>
       </c>
       <c r="D3" t="s">
+        <v>712</v>
+      </c>
+      <c r="E3" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:9">
       <c r="A4" t="s">
         <v>456</v>
       </c>
@@ -7792,10 +7811,13 @@
         <v>456</v>
       </c>
       <c r="D4" t="s">
+        <v>711</v>
+      </c>
+      <c r="E4" t="s">
         <v>457</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:9">
       <c r="A5" t="s">
         <v>458</v>
       </c>
@@ -7803,10 +7825,13 @@
         <v>458</v>
       </c>
       <c r="D5" t="s">
+        <v>712</v>
+      </c>
+      <c r="E5" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:9">
       <c r="A6" t="s">
         <v>657</v>
       </c>
@@ -7814,10 +7839,13 @@
         <v>659</v>
       </c>
       <c r="D6" t="s">
+        <v>711</v>
+      </c>
+      <c r="E6" t="s">
         <v>658</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:9">
       <c r="A7" t="s">
         <v>490</v>
       </c>
@@ -7825,10 +7853,13 @@
         <v>490</v>
       </c>
       <c r="D7" t="s">
+        <v>711</v>
+      </c>
+      <c r="E7" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:9">
       <c r="A8" t="s">
         <v>492</v>
       </c>
@@ -7836,10 +7867,13 @@
         <v>492</v>
       </c>
       <c r="D8" t="s">
+        <v>711</v>
+      </c>
+      <c r="E8" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:9">
       <c r="A9" t="s">
         <v>460</v>
       </c>
@@ -7850,22 +7884,25 @@
         <v>141</v>
       </c>
       <c r="D9" t="s">
+        <v>712</v>
+      </c>
+      <c r="E9" t="s">
         <v>461</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>678</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>677</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>698</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:9">
       <c r="A10" t="s">
         <v>462</v>
       </c>
@@ -7876,22 +7913,25 @@
         <v>141</v>
       </c>
       <c r="D10" t="s">
+        <v>712</v>
+      </c>
+      <c r="E10" t="s">
         <v>463</v>
       </c>
-      <c r="E10" t="s">
+      <c r="F10" t="s">
         <v>679</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>677</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>698</v>
       </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:9">
       <c r="A11" t="s">
         <v>464</v>
       </c>
@@ -7902,22 +7942,25 @@
         <v>141</v>
       </c>
       <c r="D11" t="s">
+        <v>712</v>
+      </c>
+      <c r="E11" t="s">
         <v>465</v>
       </c>
-      <c r="E11" t="s">
+      <c r="F11" t="s">
         <v>680</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>677</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>698</v>
       </c>
-      <c r="H11" t="s">
+      <c r="I11" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:9">
       <c r="A12" t="s">
         <v>466</v>
       </c>
@@ -7928,22 +7971,25 @@
         <v>141</v>
       </c>
       <c r="D12" t="s">
+        <v>712</v>
+      </c>
+      <c r="E12" t="s">
         <v>467</v>
       </c>
-      <c r="E12" t="s">
+      <c r="F12" t="s">
         <v>681</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>677</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>698</v>
       </c>
-      <c r="H12" t="s">
+      <c r="I12" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:9">
       <c r="A13" t="s">
         <v>468</v>
       </c>
@@ -7954,22 +8000,25 @@
         <v>141</v>
       </c>
       <c r="D13" t="s">
+        <v>712</v>
+      </c>
+      <c r="E13" t="s">
         <v>469</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>682</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>677</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>698</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:9">
       <c r="A14" t="s">
         <v>470</v>
       </c>
@@ -7980,19 +8029,22 @@
         <v>510</v>
       </c>
       <c r="D14" t="s">
+        <v>712</v>
+      </c>
+      <c r="E14" t="s">
         <v>471</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>683</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>695</v>
       </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:9">
       <c r="A15" t="s">
         <v>472</v>
       </c>
@@ -8003,19 +8055,22 @@
         <v>510</v>
       </c>
       <c r="D15" t="s">
+        <v>712</v>
+      </c>
+      <c r="E15" t="s">
         <v>473</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>684</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>696</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:9">
       <c r="A16" t="s">
         <v>474</v>
       </c>
@@ -8026,19 +8081,22 @@
         <v>510</v>
       </c>
       <c r="D16" t="s">
+        <v>712</v>
+      </c>
+      <c r="E16" t="s">
         <v>475</v>
       </c>
-      <c r="E16" t="s">
+      <c r="F16" t="s">
         <v>685</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>697</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:9">
       <c r="A17" t="s">
         <v>476</v>
       </c>
@@ -8049,16 +8107,19 @@
         <v>699</v>
       </c>
       <c r="D17" t="s">
+        <v>712</v>
+      </c>
+      <c r="E17" t="s">
         <v>477</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>686</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>689</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:9">
       <c r="A18" t="s">
         <v>478</v>
       </c>
@@ -8069,19 +8130,22 @@
         <v>509</v>
       </c>
       <c r="D18" t="s">
+        <v>712</v>
+      </c>
+      <c r="E18" t="s">
         <v>479</v>
       </c>
-      <c r="E18" t="s">
+      <c r="F18" t="s">
         <v>688</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>689</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:9">
       <c r="A19" t="s">
         <v>480</v>
       </c>
@@ -8092,19 +8156,22 @@
         <v>509</v>
       </c>
       <c r="D19" t="s">
+        <v>712</v>
+      </c>
+      <c r="E19" t="s">
         <v>481</v>
       </c>
-      <c r="E19" t="s">
+      <c r="F19" t="s">
         <v>690</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>689</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:9">
       <c r="A20" t="s">
         <v>482</v>
       </c>
@@ -8115,19 +8182,22 @@
         <v>511</v>
       </c>
       <c r="D20" t="s">
+        <v>712</v>
+      </c>
+      <c r="E20" t="s">
         <v>483</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>691</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>689</v>
       </c>
-      <c r="H20" t="s">
+      <c r="I20" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:9">
       <c r="A21" t="s">
         <v>484</v>
       </c>
@@ -8138,19 +8208,22 @@
         <v>700</v>
       </c>
       <c r="D21" t="s">
+        <v>712</v>
+      </c>
+      <c r="E21" t="s">
         <v>485</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>692</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>693</v>
       </c>
-      <c r="H21" t="s">
+      <c r="I21" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:9">
       <c r="A22" t="s">
         <v>486</v>
       </c>
@@ -8161,15 +8234,18 @@
         <v>701</v>
       </c>
       <c r="D22" t="s">
+        <v>712</v>
+      </c>
+      <c r="E22" t="s">
         <v>487</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>694</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>693</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>365</v>
       </c>
     </row>

</xml_diff>